<commit_message>
Clean commit without large zip file
</commit_message>
<xml_diff>
--- a/stats for com eng/excel files/Ch05-01.xlsx
+++ b/stats for com eng/excel files/Ch05-01.xlsx
@@ -1,23 +1,27 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10531"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10703"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/pin/Desktop/joint-repository/stats for com eng/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/pin/Desktop/joint-repository/stats for com eng/excel files/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3476AF7F-3F8D-174D-8663-E9FB21504B86}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{33117E85-D733-394B-A6F0-5D937683D650}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="600" windowWidth="24080" windowHeight="13220" activeTab="3" xr2:uid="{C748285C-19E1-4F2D-927D-6F526C53A5E8}"/>
+    <workbookView xWindow="0" yWindow="600" windowWidth="20480" windowHeight="11040" activeTab="8" xr2:uid="{C748285C-19E1-4F2D-927D-6F526C53A5E8}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="2" r:id="rId1"/>
-    <sheet name="Sheet2" sheetId="9" r:id="rId2"/>
-    <sheet name="Sheet3" sheetId="10" r:id="rId3"/>
-    <sheet name="Sheet4" sheetId="11" r:id="rId4"/>
-    <sheet name="Sheet5" sheetId="13" r:id="rId5"/>
+    <sheet name="Sheet1 practice" sheetId="14" r:id="rId2"/>
+    <sheet name="Sheet2" sheetId="9" r:id="rId3"/>
+    <sheet name="Sheet2 practice" sheetId="15" r:id="rId4"/>
+    <sheet name="Sheet3" sheetId="10" r:id="rId5"/>
+    <sheet name="Sheet3 practice" sheetId="17" r:id="rId6"/>
+    <sheet name="Sheet4" sheetId="11" r:id="rId7"/>
+    <sheet name="Sheet4 practice" sheetId="16" r:id="rId8"/>
+    <sheet name="Sheet5" sheetId="13" r:id="rId9"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -40,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="108" uniqueCount="57">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="318" uniqueCount="121">
   <si>
     <t>Parameter of Interest</t>
   </si>
@@ -280,6 +284,198 @@
   <si>
     <t>t(alpha)</t>
   </si>
+  <si>
+    <t>standard cement</t>
+  </si>
+  <si>
+    <t>cement doped with lead</t>
+  </si>
+  <si>
+    <t>n</t>
+  </si>
+  <si>
+    <t>mean</t>
+  </si>
+  <si>
+    <t>sample stdev</t>
+  </si>
+  <si>
+    <t>alpha</t>
+  </si>
+  <si>
+    <t>same pop stdev</t>
+  </si>
+  <si>
+    <t>left tail</t>
+  </si>
+  <si>
+    <t>test statistics</t>
+  </si>
+  <si>
+    <t>H0</t>
+  </si>
+  <si>
+    <t>H1</t>
+  </si>
+  <si>
+    <t>Mu1 = Mu2</t>
+  </si>
+  <si>
+    <t>Mu1 &lt; Mu2</t>
+  </si>
+  <si>
+    <t>Mu1 - Mu2 &lt; 0</t>
+  </si>
+  <si>
+    <t>Mu1 - Mu2 = 0</t>
+  </si>
+  <si>
+    <t>Pooled estimator</t>
+  </si>
+  <si>
+    <t>df</t>
+  </si>
+  <si>
+    <t>LT</t>
+  </si>
+  <si>
+    <t>critical value</t>
+  </si>
+  <si>
+    <t>accept</t>
+  </si>
+  <si>
+    <t>normal population of both types of cement likely share is similar population mean</t>
+  </si>
+  <si>
+    <t>P value</t>
+  </si>
+  <si>
+    <t>confidence interval</t>
+  </si>
+  <si>
+    <t>critical value alpha/2</t>
+  </si>
+  <si>
+    <t>critical value 1-alpha/2</t>
+  </si>
+  <si>
+    <t>lower CB</t>
+  </si>
+  <si>
+    <t>Upper CB</t>
+  </si>
+  <si>
+    <t>Formulation 1</t>
+  </si>
+  <si>
+    <t>reduce drying time</t>
+  </si>
+  <si>
+    <t>stdev 8</t>
+  </si>
+  <si>
+    <t>stdev</t>
+  </si>
+  <si>
+    <t>formulation 2</t>
+  </si>
+  <si>
+    <t>Mu1 &gt; Mu2</t>
+  </si>
+  <si>
+    <t>Mu = Mu2</t>
+  </si>
+  <si>
+    <t>RT</t>
+  </si>
+  <si>
+    <t>we have strong enough evidence to reject H0, meaning that the new formula really reduces the paint drying time</t>
+  </si>
+  <si>
+    <t>Wax 1</t>
+  </si>
+  <si>
+    <t>Wax 2</t>
+  </si>
+  <si>
+    <t>Pop stdev</t>
+  </si>
+  <si>
+    <t>Mu1 - Mu2 &gt; 0</t>
+  </si>
+  <si>
+    <t>test statistic</t>
+  </si>
+  <si>
+    <t>critical vlaue</t>
+  </si>
+  <si>
+    <t>p value</t>
+  </si>
+  <si>
+    <t>Upper bound</t>
+  </si>
+  <si>
+    <t>lower bound</t>
+  </si>
+  <si>
+    <t>Different pop variance</t>
+  </si>
+  <si>
+    <t>unknown pop variance</t>
+  </si>
+  <si>
+    <t>T test</t>
+  </si>
+  <si>
+    <t>two sample</t>
+  </si>
+  <si>
+    <t>Pheonix</t>
+  </si>
+  <si>
+    <t>Arizona</t>
+  </si>
+  <si>
+    <t>2T</t>
+  </si>
+  <si>
+    <t>variance</t>
+  </si>
+  <si>
+    <t>devided by n</t>
+  </si>
+  <si>
+    <t>2t</t>
+  </si>
+  <si>
+    <t>equal pop stdev</t>
+  </si>
+  <si>
+    <t>unknown value</t>
+  </si>
+  <si>
+    <t>catalyst 1</t>
+  </si>
+  <si>
+    <t>catalyst 2</t>
+  </si>
+  <si>
+    <t>Mu1 != Mu2</t>
+  </si>
+  <si>
+    <t>Mu1 - Mu2 != 0</t>
+  </si>
+  <si>
+    <t>Two sample t test equal pop stdev</t>
+  </si>
+  <si>
+    <t>Df</t>
+  </si>
+  <si>
+    <t>we fail to reject H0 so that means there is no difference in mean yields, catalyst 2 can be used in the test</t>
+  </si>
 </sst>
 </file>
 
@@ -289,7 +485,7 @@
     <numFmt numFmtId="164" formatCode="0.0000"/>
     <numFmt numFmtId="165" formatCode="0.00000"/>
   </numFmts>
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -316,6 +512,14 @@
       <u/>
       <sz val="11"/>
       <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -415,7 +619,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
@@ -479,6 +683,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -547,6 +754,143 @@
 </file>
 
 <file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>19050</xdr:colOff>
+      <xdr:row>7</xdr:row>
+      <xdr:rowOff>6350</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>1759184</xdr:colOff>
+      <xdr:row>14</xdr:row>
+      <xdr:rowOff>241299</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Picture 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{BD9F05ED-F5EE-9441-B1F8-D38DD73708B8}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="6115050" y="1784350"/>
+          <a:ext cx="3695934" cy="2012949"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>19</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>1507067</xdr:colOff>
+      <xdr:row>28</xdr:row>
+      <xdr:rowOff>94841</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="3" name="Picture 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{19B6DD82-949B-BB7A-A1EA-F1513C159C5E}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="4826000"/>
+          <a:ext cx="3691467" cy="2380841"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>111404</xdr:colOff>
+      <xdr:row>28</xdr:row>
+      <xdr:rowOff>89123</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>1623595</xdr:colOff>
+      <xdr:row>36</xdr:row>
+      <xdr:rowOff>83998</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="4" name="Picture 3">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{3FAF9F6A-D0CC-0AFA-172A-BBB7FA22179E}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="111404" y="7263509"/>
+          <a:ext cx="3695700" cy="2044700"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
@@ -639,7 +983,232 @@
 </xdr:wsDr>
 </file>
 
-<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/drawings/drawing4.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>19050</xdr:colOff>
+      <xdr:row>7</xdr:row>
+      <xdr:rowOff>6350</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>1762359</xdr:colOff>
+      <xdr:row>14</xdr:row>
+      <xdr:rowOff>238124</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Picture 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{1C618F33-8C69-264A-9541-2BE7C0268C26}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="6115050" y="1784350"/>
+          <a:ext cx="3699109" cy="2009774"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>19050</xdr:colOff>
+      <xdr:row>18</xdr:row>
+      <xdr:rowOff>133350</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>1787768</xdr:colOff>
+      <xdr:row>22</xdr:row>
+      <xdr:rowOff>247650</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="3" name="Picture 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{262829B5-826A-6B40-A0CF-C21BC35ECE7D}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="6115050" y="4705350"/>
+          <a:ext cx="3724518" cy="1130300"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>26</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>1139084</xdr:colOff>
+      <xdr:row>33</xdr:row>
+      <xdr:rowOff>139390</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="4" name="Picture 3">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{84964F02-D9DC-7562-A436-7CB60D8E0D3A}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="6644268"/>
+          <a:ext cx="3322864" cy="1928232"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>54207</xdr:colOff>
+      <xdr:row>33</xdr:row>
+      <xdr:rowOff>232318</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>844086</xdr:colOff>
+      <xdr:row>40</xdr:row>
+      <xdr:rowOff>88697</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="5" name="Picture 4">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{8299B0F1-DBF1-F44C-AEA3-7F0D24651D22}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId4"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="54207" y="8665428"/>
+          <a:ext cx="2973659" cy="1645220"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>10160</xdr:colOff>
+      <xdr:row>42</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>937651</xdr:colOff>
+      <xdr:row>48</xdr:row>
+      <xdr:rowOff>41484</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="6" name="Picture 5">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{5974DBEF-925E-CDB1-0E68-602CA7549A40}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId5"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="10160" y="10668000"/>
+          <a:ext cx="5072771" cy="1565484"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing5.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
@@ -732,7 +1301,188 @@
 </xdr:wsDr>
 </file>
 
-<file path=xl/drawings/drawing4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/drawings/drawing6.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>641350</xdr:colOff>
+      <xdr:row>5</xdr:row>
+      <xdr:rowOff>76201</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>10690</xdr:colOff>
+      <xdr:row>8</xdr:row>
+      <xdr:rowOff>104776</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Picture 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{74DAD30B-2540-4945-A7EE-BC4B49815D4B}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="4781550" y="1346201"/>
+          <a:ext cx="3280940" cy="790575"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>29881</xdr:colOff>
+      <xdr:row>8</xdr:row>
+      <xdr:rowOff>179294</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>1706468</xdr:colOff>
+      <xdr:row>15</xdr:row>
+      <xdr:rowOff>65543</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="3" name="Picture 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{25197EC2-4565-2147-9076-004E9E3F0EDA}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="6125881" y="2211294"/>
+          <a:ext cx="3632387" cy="1664249"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>25</xdr:row>
+      <xdr:rowOff>33866</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>1929207</xdr:colOff>
+      <xdr:row>38</xdr:row>
+      <xdr:rowOff>50799</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="4" name="Picture 3">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{18BA0060-A0E0-6B6F-D064-E765B63FBC4E}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="6383866"/>
+          <a:ext cx="4113607" cy="3318933"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>554836</xdr:colOff>
+      <xdr:row>27</xdr:row>
+      <xdr:rowOff>67733</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>875118</xdr:colOff>
+      <xdr:row>38</xdr:row>
+      <xdr:rowOff>190499</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="5" name="Picture 4">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{9EA99A30-A583-5134-E456-C1B2A0E8A64A}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId4"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="10562436" y="6925733"/>
+          <a:ext cx="4231882" cy="2916766"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing7.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
@@ -858,6 +1608,544 @@
         <a:xfrm>
           <a:off x="6105181" y="4796928"/>
           <a:ext cx="7772400" cy="4556234"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing8.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>36146</xdr:colOff>
+      <xdr:row>7</xdr:row>
+      <xdr:rowOff>25889</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>1790073</xdr:colOff>
+      <xdr:row>9</xdr:row>
+      <xdr:rowOff>238125</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Picture 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{3616D37B-B3EC-7D42-BF97-98FB01C3873D}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="6132146" y="1803889"/>
+          <a:ext cx="3709727" cy="720236"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>29882</xdr:colOff>
+      <xdr:row>14</xdr:row>
+      <xdr:rowOff>37354</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>1778264</xdr:colOff>
+      <xdr:row>16</xdr:row>
+      <xdr:rowOff>235885</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="3" name="Picture 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{F106FBAF-C17E-3246-8BB0-71B2218C94B5}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="6125882" y="3593354"/>
+          <a:ext cx="3704182" cy="706531"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>19</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>1896738</xdr:colOff>
+      <xdr:row>37</xdr:row>
+      <xdr:rowOff>11776</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="4" name="Picture 3">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{E086B16F-5CE9-1149-ACED-4A338AA5ACDA}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="6096000" y="4826000"/>
+          <a:ext cx="7764138" cy="4583776"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>40</xdr:row>
+      <xdr:rowOff>60960</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>1835753</xdr:colOff>
+      <xdr:row>56</xdr:row>
+      <xdr:rowOff>228600</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="5" name="Picture 4">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{4A02301C-0FA0-2944-C05A-A91870F2EBB2}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId4"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="10220960"/>
+          <a:ext cx="5981033" cy="4231640"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>233680</xdr:colOff>
+      <xdr:row>57</xdr:row>
+      <xdr:rowOff>233680</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>1778000</xdr:colOff>
+      <xdr:row>66</xdr:row>
+      <xdr:rowOff>106680</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="6" name="Picture 5">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{9ED59D14-0074-41ED-74D1-C015241D684D}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId5"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="233680" y="14711680"/>
+          <a:ext cx="5689600" cy="2159000"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>52</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>1760220</xdr:colOff>
+      <xdr:row>54</xdr:row>
+      <xdr:rowOff>228600</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="7" name="Picture 6">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{89CBA75C-CE57-DC8B-4B9C-C3169DD2A23F}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId6"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="11988800" y="13208000"/>
+          <a:ext cx="3721100" cy="736600"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>56</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>1747520</xdr:colOff>
+      <xdr:row>58</xdr:row>
+      <xdr:rowOff>215900</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="8" name="Picture 7">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{CFC92A76-A3DC-C129-2B3B-94B53F99C978}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId7"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="11988800" y="14224000"/>
+          <a:ext cx="3708400" cy="723900"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>20320</xdr:colOff>
+      <xdr:row>61</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>1910080</xdr:colOff>
+      <xdr:row>72</xdr:row>
+      <xdr:rowOff>77470</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="9" name="Picture 8">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{8C7CF182-CDA3-050B-C8B4-21041A0BB9DA}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId8"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="12009120" y="15494000"/>
+          <a:ext cx="7772400" cy="2871470"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing9.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>313267</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>237068</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>93133</xdr:colOff>
+      <xdr:row>11</xdr:row>
+      <xdr:rowOff>151852</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Picture 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{69F82A00-C873-F264-E4D3-A1110FCC15C5}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="8365067" y="237068"/>
+          <a:ext cx="3691466" cy="2708784"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>1905000</xdr:colOff>
+      <xdr:row>7</xdr:row>
+      <xdr:rowOff>110067</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>1282700</xdr:colOff>
+      <xdr:row>10</xdr:row>
+      <xdr:rowOff>160867</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="3" name="Picture 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{36A28E6A-A4B6-2356-3384-61412CD9DCCA}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="19735800" y="1888067"/>
+          <a:ext cx="3289300" cy="812800"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>11</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>1676400</xdr:colOff>
+      <xdr:row>17</xdr:row>
+      <xdr:rowOff>165100</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="4" name="Picture 3">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{9C127407-F3E1-95FA-4360-C3DA9A21D348}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="19786600" y="2794000"/>
+          <a:ext cx="3632200" cy="1689100"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>50800</xdr:colOff>
+      <xdr:row>18</xdr:row>
+      <xdr:rowOff>54085</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>12</xdr:col>
+      <xdr:colOff>1011767</xdr:colOff>
+      <xdr:row>28</xdr:row>
+      <xdr:rowOff>21166</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="5" name="Picture 4">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{A9EC130E-C076-646A-4452-45E5352DE208}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId4"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="19837400" y="4626085"/>
+          <a:ext cx="4872567" cy="2507081"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1355,6 +2643,324 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8986DDF8-8A4E-6E47-826C-4C2957901B34}">
+  <dimension ref="A1:F34"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="25.6640625" defaultRowHeight="20" customHeight="1" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="28.6640625" style="3" customWidth="1"/>
+    <col min="2" max="2" width="25.6640625" style="1"/>
+    <col min="3" max="3" width="25.6640625" style="2"/>
+    <col min="4" max="16384" width="25.6640625" style="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" s="14" customFormat="1" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A1" s="13" t="s">
+        <v>8</v>
+      </c>
+      <c r="C1" s="15"/>
+    </row>
+    <row r="2" spans="1:4" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A2" s="1"/>
+      <c r="B2" s="2"/>
+      <c r="C2" s="1"/>
+    </row>
+    <row r="3" spans="1:4" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A3" s="11" t="s">
+        <v>11</v>
+      </c>
+      <c r="B3" s="5">
+        <v>10</v>
+      </c>
+      <c r="C3" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="D3" s="5">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A4" s="11" t="s">
+        <v>9</v>
+      </c>
+      <c r="B4" s="5">
+        <v>121</v>
+      </c>
+      <c r="C4" s="11" t="s">
+        <v>10</v>
+      </c>
+      <c r="D4" s="5">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A5" s="11" t="s">
+        <v>14</v>
+      </c>
+      <c r="B5" s="5">
+        <v>8</v>
+      </c>
+      <c r="C5" s="11" t="s">
+        <v>15</v>
+      </c>
+      <c r="D5" s="5">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A6" s="12"/>
+      <c r="C6" s="1"/>
+    </row>
+    <row r="7" spans="1:4" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A7" s="1"/>
+      <c r="B7" s="6"/>
+      <c r="C7" s="1" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A8" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="B8" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="C8" s="1"/>
+    </row>
+    <row r="9" spans="1:4" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A9" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="B9" s="19" t="s">
+        <v>33</v>
+      </c>
+      <c r="C9" s="1"/>
+    </row>
+    <row r="10" spans="1:4" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A10" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="B10" s="19" t="s">
+        <v>34</v>
+      </c>
+      <c r="C10" s="1"/>
+    </row>
+    <row r="11" spans="1:4" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A11" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="B11" s="7">
+        <v>0.05</v>
+      </c>
+      <c r="C11" s="1"/>
+    </row>
+    <row r="12" spans="1:4" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A12" s="20" t="s">
+        <v>3</v>
+      </c>
+      <c r="B12" s="7" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A13" s="21"/>
+      <c r="B13" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C13" s="1"/>
+    </row>
+    <row r="14" spans="1:4" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A14" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="B14" s="5">
+        <f>(B4-D4)/(SQRT(POWER(B5,2)/B3+POWER(D5,2)/D3))</f>
+        <v>2.5155764746872635</v>
+      </c>
+      <c r="C14" s="1"/>
+    </row>
+    <row r="15" spans="1:4" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A15" s="8" t="s">
+        <v>36</v>
+      </c>
+      <c r="B15" s="9">
+        <f>_xlfn.NORM.S.INV(1-B11)</f>
+        <v>1.6448536269514715</v>
+      </c>
+      <c r="C15" s="1"/>
+    </row>
+    <row r="16" spans="1:4" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A16" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="B16" s="9">
+        <f>1-_xlfn.NORM.S.DIST(B14, TRUE)</f>
+        <v>5.9418946210736401E-3</v>
+      </c>
+      <c r="C16" s="1"/>
+    </row>
+    <row r="17" spans="1:6" ht="20" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="1"/>
+      <c r="B17" s="3"/>
+      <c r="C17" s="1"/>
+    </row>
+    <row r="18" spans="1:6" ht="20" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A18" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B18" s="10" t="s">
+        <v>39</v>
+      </c>
+      <c r="C18" s="1"/>
+    </row>
+    <row r="19" spans="1:6" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A19" s="1"/>
+      <c r="B19" s="2"/>
+      <c r="C19" s="1"/>
+    </row>
+    <row r="20" spans="1:6" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A20" s="1"/>
+      <c r="B20" s="2"/>
+      <c r="C20" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="D20" s="1" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="C21" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="E21" s="1" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="C22" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="D22" s="1">
+        <v>121</v>
+      </c>
+      <c r="F22" s="1">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="C23" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="D23" s="1">
+        <v>10</v>
+      </c>
+      <c r="F23" s="1">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="C24" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="D24" s="1">
+        <v>8</v>
+      </c>
+      <c r="F24" s="1">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="C25" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="D25" s="1">
+        <v>0.05</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="C26" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="D26" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="E26" s="1" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="C27" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="D27" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="E27" s="1" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="C28" s="2" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="C29" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="D29" s="1">
+        <f>_xlfn.NORM.S.DIST(1-D25, TRUE)</f>
+        <v>0.82894387369151812</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="C30" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="D30" s="1">
+        <f>(D22-F22)/SQRT(D24^2/D23+F24^2/F23)</f>
+        <v>2.5155764746872635</v>
+      </c>
+      <c r="E30" s="1" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="C31" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="D31" s="1">
+        <f>D25</f>
+        <v>0.05</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="C32" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="D32" s="1">
+        <f>1-_xlfn.NORM.S.DIST(D30, TRUE)</f>
+        <v>5.9418946210736401E-3</v>
+      </c>
+      <c r="E32" s="1" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="34" spans="3:3" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="C34" s="2" t="s">
+        <v>92</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A12:A13"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+  <drawing r:id="rId2"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{77FCDD7B-BBAF-4196-8F35-C57A6D7C449A}">
   <dimension ref="A1:D23"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="25.6640625" defaultRowHeight="20" customHeight="1" x14ac:dyDescent="0.2"/>
@@ -1564,7 +3170,344 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{41B711FA-EE11-044D-AF50-DFBB8E1C25EB}">
+  <dimension ref="A1:E42"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="25.6640625" defaultRowHeight="20" customHeight="1" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="28.6640625" style="3" customWidth="1"/>
+    <col min="2" max="2" width="25.6640625" style="1"/>
+    <col min="3" max="3" width="25.6640625" style="2"/>
+    <col min="4" max="16384" width="25.6640625" style="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A1" s="13" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A2" s="1"/>
+      <c r="B2" s="2"/>
+      <c r="C2" s="1"/>
+    </row>
+    <row r="3" spans="1:4" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A3" s="11" t="s">
+        <v>11</v>
+      </c>
+      <c r="B3" s="5">
+        <v>20</v>
+      </c>
+      <c r="C3" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="D3" s="5">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A4" s="11" t="s">
+        <v>9</v>
+      </c>
+      <c r="B4" s="5">
+        <v>3</v>
+      </c>
+      <c r="C4" s="11" t="s">
+        <v>10</v>
+      </c>
+      <c r="D4" s="5">
+        <v>2.9</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A5" s="11" t="s">
+        <v>14</v>
+      </c>
+      <c r="B5" s="5">
+        <v>0.33</v>
+      </c>
+      <c r="C5" s="11" t="s">
+        <v>15</v>
+      </c>
+      <c r="D5" s="5">
+        <v>0.36</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A6" s="12"/>
+      <c r="C6" s="1"/>
+    </row>
+    <row r="7" spans="1:4" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A7" s="1"/>
+      <c r="B7" s="6"/>
+      <c r="C7" s="1"/>
+    </row>
+    <row r="8" spans="1:4" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A8" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="B8" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="C8" s="1"/>
+    </row>
+    <row r="9" spans="1:4" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A9" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="B9" s="7" t="s">
+        <v>40</v>
+      </c>
+      <c r="C9" s="1"/>
+    </row>
+    <row r="10" spans="1:4" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A10" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="B10" s="7" t="s">
+        <v>44</v>
+      </c>
+      <c r="C10" s="1"/>
+    </row>
+    <row r="11" spans="1:4" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A11" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="B11" s="7">
+        <v>0.05</v>
+      </c>
+      <c r="C11" s="1"/>
+    </row>
+    <row r="12" spans="1:4" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A12" s="20" t="s">
+        <v>3</v>
+      </c>
+      <c r="B12" s="7" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A13" s="21"/>
+      <c r="B13" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C13" s="1"/>
+    </row>
+    <row r="14" spans="1:4" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A14" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="B14" s="5">
+        <f>(B4-D4-0)/SQRT(POWER(B5,2)/B3+POWER(D5,2)/D3)</f>
+        <v>0.91573709299126105</v>
+      </c>
+      <c r="C14" s="1"/>
+    </row>
+    <row r="15" spans="1:4" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A15" s="8" t="s">
+        <v>43</v>
+      </c>
+      <c r="B15" s="9">
+        <f>_xlfn.NORM.S.INV(1-B11)</f>
+        <v>1.6448536269514715</v>
+      </c>
+      <c r="C15" s="1"/>
+    </row>
+    <row r="16" spans="1:4" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A16" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="B16" s="9">
+        <f>1-_xlfn.NORM.S.DIST(B14,TRUE)</f>
+        <v>0.17990240246271461</v>
+      </c>
+      <c r="C16" s="1"/>
+    </row>
+    <row r="17" spans="1:5" ht="20" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="1"/>
+      <c r="B17" s="3"/>
+      <c r="C17" s="1"/>
+    </row>
+    <row r="18" spans="1:5" ht="20" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A18" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B18" s="10" t="s">
+        <v>45</v>
+      </c>
+      <c r="C18" s="1"/>
+    </row>
+    <row r="19" spans="1:5" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A19" s="1"/>
+      <c r="B19" s="2"/>
+      <c r="C19" s="1"/>
+    </row>
+    <row r="20" spans="1:5" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A20" s="1"/>
+      <c r="B20" s="2"/>
+      <c r="C20" s="1"/>
+    </row>
+    <row r="21" spans="1:5" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A21" s="3" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A22" s="16" t="s">
+        <v>17</v>
+      </c>
+      <c r="B22" s="17">
+        <f>B4-D4-_xlfn.NORM.S.INV(1-B11/2)*SQRT(POWER(B5,2)/B3+POWER(D5,2)/D3)</f>
+        <v>-0.11403129779725529</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A23" s="16" t="s">
+        <v>18</v>
+      </c>
+      <c r="B23" s="17">
+        <f>B4-D4+_xlfn.NORM.S.INV(1-B11/2)*SQRT(POWER(B5,2)/B3+POWER(D5,2)/D3)</f>
+        <v>0.31403129779725547</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D28" s="2" t="s">
+        <v>93</v>
+      </c>
+      <c r="E28" s="1" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="C29" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="D29" s="1">
+        <v>20</v>
+      </c>
+      <c r="E29" s="1">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="C30" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="D30" s="1">
+        <v>3</v>
+      </c>
+      <c r="E30" s="1">
+        <v>2.9</v>
+      </c>
+    </row>
+    <row r="31" spans="1:5" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="C31" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="D31" s="1">
+        <v>0.33</v>
+      </c>
+      <c r="E31" s="1">
+        <v>0.36</v>
+      </c>
+    </row>
+    <row r="33" spans="3:5" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="C33" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="D33" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="E33" s="1" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="34" spans="3:5" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="C34" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="D34" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="E34" s="1" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="35" spans="3:5" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="C35" s="2" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="36" spans="3:5" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="C36" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="D36" s="1">
+        <f>_xlfn.NORM.S.INV(1-D38)</f>
+        <v>1.6448536269514715</v>
+      </c>
+    </row>
+    <row r="37" spans="3:5" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="C37" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="D37" s="1">
+        <f>(D30-E30)/SQRT(D31^2/D29+E31^2/E29)</f>
+        <v>0.91573709299126105</v>
+      </c>
+      <c r="E37" s="1" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="38" spans="3:5" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="C38" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="D38" s="1">
+        <v>0.05</v>
+      </c>
+    </row>
+    <row r="39" spans="3:5" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="C39" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="D39" s="1">
+        <f>1-_xlfn.NORM.S.DIST(D37, TRUE)</f>
+        <v>0.17990240246271461</v>
+      </c>
+      <c r="E39" s="1" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="41" spans="3:5" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="C41" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="D41" s="1">
+        <f>D30-E30 +_xlfn.NORM.S.INV(1-D38/2) *SQRT(D31^2/D29+E31^2/E29)</f>
+        <v>0.31403129779725547</v>
+      </c>
+    </row>
+    <row r="42" spans="3:5" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="C42" s="2" t="s">
+        <v>101</v>
+      </c>
+      <c r="D42" s="1">
+        <f>D30-E30 -_xlfn.NORM.S.INV(1-D38/2) *SQRT(D31^2/D29+E31^2/E29)</f>
+        <v>-0.11403129779725529</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A12:A13"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+  <drawing r:id="rId2"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FD0529F6-0578-427D-894E-246593E33DA1}">
   <dimension ref="A1:D22"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="25.6640625" defaultRowHeight="20" customHeight="1" x14ac:dyDescent="0.2"/>
@@ -1773,7 +3716,371 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4F57E6D1-4DB3-7E4F-96F9-FC5036F2A182}">
+  <dimension ref="A1:G42"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="25.6640625" defaultRowHeight="20" customHeight="1" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="28.6640625" style="3" customWidth="1"/>
+    <col min="2" max="2" width="25.6640625" style="1"/>
+    <col min="3" max="3" width="25.6640625" style="2"/>
+    <col min="4" max="16384" width="25.6640625" style="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" s="14" customFormat="1" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A1" s="13" t="s">
+        <v>20</v>
+      </c>
+      <c r="C1" s="15"/>
+    </row>
+    <row r="2" spans="1:4" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A2" s="1"/>
+      <c r="B2" s="2"/>
+      <c r="C2" s="1"/>
+    </row>
+    <row r="3" spans="1:4" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A3" s="11" t="s">
+        <v>11</v>
+      </c>
+      <c r="B3" s="5">
+        <v>8</v>
+      </c>
+      <c r="C3" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="D3" s="5">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A4" s="11" t="s">
+        <v>9</v>
+      </c>
+      <c r="B4" s="5">
+        <v>92.254999999999995</v>
+      </c>
+      <c r="C4" s="11" t="s">
+        <v>10</v>
+      </c>
+      <c r="D4" s="5">
+        <v>92.733000000000004</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A5" s="11" t="s">
+        <v>21</v>
+      </c>
+      <c r="B5" s="5">
+        <v>2.39</v>
+      </c>
+      <c r="C5" s="11" t="s">
+        <v>22</v>
+      </c>
+      <c r="D5" s="5">
+        <v>2.98</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A6" s="11" t="s">
+        <v>23</v>
+      </c>
+      <c r="B6" s="5">
+        <f>((B3-1)*POWER(B5,2) + (D3-1)*POWER(D5,2))/(B3+D3-2)</f>
+        <v>7.2962500000000006</v>
+      </c>
+      <c r="C6" s="1"/>
+    </row>
+    <row r="7" spans="1:4" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A7" s="1"/>
+      <c r="B7" s="6"/>
+      <c r="C7" s="1"/>
+    </row>
+    <row r="8" spans="1:4" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A8" s="1"/>
+      <c r="B8" s="6"/>
+      <c r="C8" s="1"/>
+    </row>
+    <row r="9" spans="1:4" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A9" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="B9" s="7" t="s">
+        <v>46</v>
+      </c>
+      <c r="C9" s="1"/>
+    </row>
+    <row r="10" spans="1:4" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A10" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="B10" s="7" t="s">
+        <v>47</v>
+      </c>
+      <c r="C10" s="1"/>
+    </row>
+    <row r="11" spans="1:4" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A11" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="B11" s="7" t="s">
+        <v>48</v>
+      </c>
+      <c r="C11" s="1"/>
+    </row>
+    <row r="12" spans="1:4" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A12" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="B12" s="7">
+        <v>0.05</v>
+      </c>
+      <c r="C12" s="1"/>
+    </row>
+    <row r="13" spans="1:4" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A13" s="20" t="s">
+        <v>3</v>
+      </c>
+      <c r="B13" s="7" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A14" s="21"/>
+      <c r="B14" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C14" s="1"/>
+    </row>
+    <row r="15" spans="1:4" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A15" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="B15" s="5">
+        <f>(B4-D4-0)/(SQRT(B6)*SQRT(1/B3+1/D3))</f>
+        <v>-0.35392239087555299</v>
+      </c>
+      <c r="C15" s="1"/>
+    </row>
+    <row r="16" spans="1:4" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A16" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="B16" s="18">
+        <f>B3+D3-2</f>
+        <v>14</v>
+      </c>
+      <c r="C16" s="1"/>
+    </row>
+    <row r="17" spans="1:7" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A17" s="8" t="s">
+        <v>50</v>
+      </c>
+      <c r="B17" s="9">
+        <f>_xlfn.T.INV(1-B12/2, B16)</f>
+        <v>2.1447866879178035</v>
+      </c>
+      <c r="C17" s="1"/>
+    </row>
+    <row r="18" spans="1:7" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A18" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="B18" s="9">
+        <f>_xlfn.T.DIST.2T(ABS(B15),B16)</f>
+        <v>0.72867055309702922</v>
+      </c>
+      <c r="C18" s="1"/>
+    </row>
+    <row r="19" spans="1:7" ht="20" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="1"/>
+      <c r="B19" s="3"/>
+      <c r="C19" s="1"/>
+    </row>
+    <row r="20" spans="1:7" ht="20" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A20" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B20" s="10" t="s">
+        <v>52</v>
+      </c>
+      <c r="C20" s="1"/>
+    </row>
+    <row r="21" spans="1:7" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A21" s="1"/>
+      <c r="B21" s="2"/>
+      <c r="C21" s="1"/>
+    </row>
+    <row r="22" spans="1:7" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A22" s="1"/>
+      <c r="B22" s="2"/>
+      <c r="C22" s="1"/>
+    </row>
+    <row r="24" spans="1:7" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D24" s="1" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D25" s="1" t="s">
+        <v>112</v>
+      </c>
+      <c r="E25" s="1" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D26" s="1" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D27" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="E27" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="G27" s="22"/>
+    </row>
+    <row r="28" spans="1:7" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="C28" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="D28" s="1">
+        <v>8</v>
+      </c>
+      <c r="E28" s="1">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="C29" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="D29" s="1">
+        <v>92.254999999999995</v>
+      </c>
+      <c r="E29" s="1">
+        <v>92.733000000000004</v>
+      </c>
+    </row>
+    <row r="30" spans="1:7" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="C30" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="D30" s="1">
+        <v>2.39</v>
+      </c>
+      <c r="E30" s="1">
+        <v>2.98</v>
+      </c>
+    </row>
+    <row r="32" spans="1:7" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="C32" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="D32" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="E32" s="1" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="33" spans="3:5" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="C33" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="D33" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="E33" s="1" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="34" spans="3:5" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="C34" s="2" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="35" spans="3:5" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="C35" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="D35" s="1">
+        <f>((D28-1)*D30^2+(E28-1)*E30^2)/(D28+E28-2)</f>
+        <v>7.2962500000000006</v>
+      </c>
+    </row>
+    <row r="36" spans="3:5" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="C36" s="2" t="s">
+        <v>119</v>
+      </c>
+      <c r="D36" s="1">
+        <f>D28+E28-2</f>
+        <v>14</v>
+      </c>
+    </row>
+    <row r="37" spans="3:5" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="C37" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="D37" s="1">
+        <f>_xlfn.T.INV(1-D39/2, D36)</f>
+        <v>2.1447866879178035</v>
+      </c>
+      <c r="E37" s="1">
+        <f>_xlfn.T.INV(D39/2, D36)</f>
+        <v>-2.1447866879178044</v>
+      </c>
+    </row>
+    <row r="38" spans="3:5" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="C38" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="D38" s="1">
+        <f>(D29-E29)/(D35*SQRT(1/D28+1/E28))</f>
+        <v>-0.13102621209525678</v>
+      </c>
+      <c r="E38" s="1" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="39" spans="3:5" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="C39" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="D39" s="1">
+        <v>0.05</v>
+      </c>
+    </row>
+    <row r="40" spans="3:5" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="C40" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="D40" s="1">
+        <f>2*(1-_xlfn.T.DIST(ABS(D38), D36, TRUE))</f>
+        <v>0.89761879173448733</v>
+      </c>
+      <c r="E40" s="1" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="42" spans="3:5" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="C42" s="2" t="s">
+        <v>120</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A13:A14"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+  <drawing r:id="rId2"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C3FCE472-BD82-4C73-808A-B57CB6B83248}">
   <dimension ref="A1:D21"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="25.6640625" defaultRowHeight="20" customHeight="1" x14ac:dyDescent="0.2"/>
@@ -1972,9 +4279,346 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2E9D73D5-14DF-B94A-8A71-40162FF03155}">
+  <dimension ref="A1:F59"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="25.6640625" defaultRowHeight="20" customHeight="1" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="28.6640625" style="3" customWidth="1"/>
+    <col min="2" max="2" width="25.6640625" style="1"/>
+    <col min="3" max="3" width="25.6640625" style="2" customWidth="1"/>
+    <col min="4" max="16384" width="25.6640625" style="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" s="14" customFormat="1" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A1" s="13" t="s">
+        <v>25</v>
+      </c>
+      <c r="C1" s="15"/>
+    </row>
+    <row r="2" spans="1:4" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A2" s="1"/>
+      <c r="B2" s="2"/>
+      <c r="C2" s="1"/>
+    </row>
+    <row r="3" spans="1:4" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A3" s="11" t="s">
+        <v>11</v>
+      </c>
+      <c r="B3" s="5">
+        <v>10</v>
+      </c>
+      <c r="C3" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="D3" s="5">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A4" s="11" t="s">
+        <v>9</v>
+      </c>
+      <c r="B4" s="5">
+        <v>12.5</v>
+      </c>
+      <c r="C4" s="11" t="s">
+        <v>10</v>
+      </c>
+      <c r="D4" s="5">
+        <v>27.5</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A5" s="11" t="s">
+        <v>21</v>
+      </c>
+      <c r="B5" s="5">
+        <v>7.63</v>
+      </c>
+      <c r="C5" s="11" t="s">
+        <v>22</v>
+      </c>
+      <c r="D5" s="5">
+        <v>15.3</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A6" s="1"/>
+      <c r="B6" s="6"/>
+      <c r="C6" s="1"/>
+    </row>
+    <row r="7" spans="1:4" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A7" s="1"/>
+      <c r="B7" s="6"/>
+      <c r="C7" s="1"/>
+    </row>
+    <row r="8" spans="1:4" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A8" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="B8" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="C8" s="1"/>
+    </row>
+    <row r="9" spans="1:4" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A9" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="B9" s="7" t="s">
+        <v>54</v>
+      </c>
+      <c r="C9" s="1"/>
+    </row>
+    <row r="10" spans="1:4" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A10" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="B10" s="7" t="s">
+        <v>48</v>
+      </c>
+      <c r="C10" s="1"/>
+    </row>
+    <row r="11" spans="1:4" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A11" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="B11" s="7">
+        <v>0.05</v>
+      </c>
+      <c r="C11" s="1"/>
+    </row>
+    <row r="12" spans="1:4" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A12" s="20" t="s">
+        <v>3</v>
+      </c>
+      <c r="B12" s="7" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A13" s="21"/>
+      <c r="B13" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C13" s="1"/>
+    </row>
+    <row r="14" spans="1:4" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A14" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="B14" s="5">
+        <f>(B4-D4-0)/SQRT(POWER(B5,2)/B3+POWER(D5,2)/D3)</f>
+        <v>-2.7744169270368957</v>
+      </c>
+      <c r="C14" s="1"/>
+    </row>
+    <row r="15" spans="1:4" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A15" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="B15" s="18">
+        <f>POWER((POWER(B5,2)/B3+POWER(D5,2)/D3),2)/(POWER(POWER(B5,2)/B3,2)/(B3-1)+POWER((POWER(D5,2)/D3),2)/(D3-1))</f>
+        <v>13.215760901884211</v>
+      </c>
+      <c r="C15" s="1"/>
+    </row>
+    <row r="16" spans="1:4" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A16" s="8" t="s">
+        <v>56</v>
+      </c>
+      <c r="B16" s="9">
+        <f>_xlfn.T.INV(1-B11/2, B15)</f>
+        <v>2.1603686564627917</v>
+      </c>
+      <c r="C16" s="1"/>
+    </row>
+    <row r="17" spans="1:3" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A17" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="B17" s="9">
+        <f>_xlfn.T.DIST.2T(ABS(B14),B15)</f>
+        <v>1.5783688581557809E-2</v>
+      </c>
+      <c r="C17" s="1"/>
+    </row>
+    <row r="18" spans="1:3" ht="20" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A18" s="1"/>
+      <c r="B18" s="3"/>
+      <c r="C18" s="1"/>
+    </row>
+    <row r="19" spans="1:3" ht="20" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B19" s="10" t="s">
+        <v>37</v>
+      </c>
+      <c r="C19" s="1"/>
+    </row>
+    <row r="20" spans="1:3" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A20" s="1"/>
+      <c r="B20" s="2"/>
+      <c r="C20" s="1"/>
+    </row>
+    <row r="21" spans="1:3" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A21" s="1"/>
+      <c r="B21" s="2"/>
+      <c r="C21" s="1"/>
+    </row>
+    <row r="46" spans="5:6" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="E46" s="1" t="s">
+        <v>102</v>
+      </c>
+      <c r="F46" s="1" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="47" spans="5:6" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="E47" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="F47" s="1" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="48" spans="5:6" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="E48" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="F48" s="1" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="49" spans="4:6" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D49" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="E49" s="1">
+        <v>10</v>
+      </c>
+      <c r="F49" s="1">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="50" spans="4:6" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D50" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="E50" s="1">
+        <v>12.5</v>
+      </c>
+      <c r="F50" s="1">
+        <v>27.5</v>
+      </c>
+    </row>
+    <row r="51" spans="4:6" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D51" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="E51" s="1">
+        <v>7.63</v>
+      </c>
+      <c r="F51" s="1">
+        <v>15.3</v>
+      </c>
+    </row>
+    <row r="52" spans="4:6" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D52" s="1" t="s">
+        <v>109</v>
+      </c>
+      <c r="E52" s="1">
+        <f>E51^2</f>
+        <v>58.216899999999995</v>
+      </c>
+      <c r="F52" s="1">
+        <f>F51^2</f>
+        <v>234.09000000000003</v>
+      </c>
+    </row>
+    <row r="53" spans="4:6" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D53" s="1" t="s">
+        <v>110</v>
+      </c>
+      <c r="E53" s="1">
+        <f>E52/E49</f>
+        <v>5.8216899999999994</v>
+      </c>
+      <c r="F53" s="1">
+        <f>F52/F49</f>
+        <v>23.409000000000002</v>
+      </c>
+    </row>
+    <row r="54" spans="4:6" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D54" s="1" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="55" spans="4:6" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D55" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="E55" s="1">
+        <f>(E53+F53)^2/((E53^2/(E49-1))+(F53^2/(F49-1)))</f>
+        <v>13.215760901884211</v>
+      </c>
+    </row>
+    <row r="56" spans="4:6" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D56" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="E56" s="1">
+        <f>_xlfn.T.INV(1-E58/2, E55)</f>
+        <v>2.1603686564627917</v>
+      </c>
+    </row>
+    <row r="57" spans="4:6" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D57" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="E57" s="1">
+        <f>(E50-F50)/SQRT(E51^2/E49+F51^2/F49)</f>
+        <v>-2.7744169270368957</v>
+      </c>
+      <c r="F57" s="1" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="58" spans="4:6" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D58" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="E58" s="1">
+        <v>0.05</v>
+      </c>
+    </row>
+    <row r="59" spans="4:6" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D59" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="E59" s="1">
+        <f>2*(1-_xlfn.T.DIST(ABS(E57), E55, TRUE))</f>
+        <v>1.5783688581557875E-2</v>
+      </c>
+      <c r="F59" s="1" t="s">
+        <v>37</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A12:A13"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+  <drawing r:id="rId2"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3890BDFB-1267-4BC8-8BC6-D9ABB7AF06E9}">
-  <dimension ref="A1:D13"/>
+  <dimension ref="A1:K28"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="25.6640625" defaultRowHeight="20" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="28.6640625" style="3" customWidth="1"/>
@@ -1983,18 +4627,18 @@
     <col min="4" max="16384" width="25.6640625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" s="14" customFormat="1" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:11" s="14" customFormat="1" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="13" t="s">
         <v>28</v>
       </c>
       <c r="C1" s="15"/>
     </row>
-    <row r="2" spans="1:4" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:11" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="1"/>
       <c r="B2" s="2"/>
       <c r="C2" s="1"/>
     </row>
-    <row r="3" spans="1:4" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:11" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="11" t="s">
         <v>11</v>
       </c>
@@ -2004,7 +4648,7 @@
       </c>
       <c r="D3" s="5"/>
     </row>
-    <row r="4" spans="1:4" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:11" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="11" t="s">
         <v>9</v>
       </c>
@@ -2013,8 +4657,17 @@
         <v>10</v>
       </c>
       <c r="D4" s="5"/>
-    </row>
-    <row r="5" spans="1:4" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="G4" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="H4" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="J4" s="1" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="11" t="s">
         <v>21</v>
       </c>
@@ -2023,61 +4676,225 @@
         <v>22</v>
       </c>
       <c r="D5" s="5"/>
-    </row>
-    <row r="6" spans="1:4" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="G5" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="H5" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="I5" s="1">
+        <v>10</v>
+      </c>
+      <c r="K5" s="1">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="11" t="s">
         <v>23</v>
       </c>
       <c r="B6" s="5"/>
       <c r="C6" s="1"/>
-    </row>
-    <row r="7" spans="1:4" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="H6" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="I6" s="1">
+        <v>90</v>
+      </c>
+      <c r="K6" s="1">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="11" t="s">
         <v>29</v>
       </c>
       <c r="B7" s="5"/>
       <c r="C7" s="1"/>
-    </row>
-    <row r="8" spans="1:4" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="H7" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="I7" s="1">
+        <v>5</v>
+      </c>
+      <c r="K7" s="1">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="11" t="s">
         <v>24</v>
       </c>
       <c r="B8" s="5"/>
       <c r="C8" s="1"/>
     </row>
-    <row r="9" spans="1:4" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:11" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="1"/>
       <c r="B9" s="2"/>
       <c r="C9" s="1"/>
-    </row>
-    <row r="10" spans="1:4" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="H9" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="I9" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="J9" s="1" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="1" t="s">
         <v>30</v>
       </c>
       <c r="B10" s="6"/>
       <c r="C10" s="1"/>
-    </row>
-    <row r="11" spans="1:4" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="H10" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="I10" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="J10" s="1" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="11" spans="1:11" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="11" t="s">
         <v>31</v>
       </c>
       <c r="B11" s="5"/>
       <c r="C11" s="1"/>
     </row>
-    <row r="12" spans="1:4" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:11" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="11" t="s">
         <v>32</v>
       </c>
       <c r="B12" s="5"/>
       <c r="C12" s="1"/>
-    </row>
-    <row r="13" spans="1:4" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="H12" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="I12" s="1">
+        <v>0.05</v>
+      </c>
+    </row>
+    <row r="13" spans="1:11" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="1"/>
       <c r="B13" s="2"/>
       <c r="C13" s="1"/>
+      <c r="H13" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="I13" s="1">
+        <f>((I5-1)*I7^2+(K5-1)*K7^2)/(I5+K5-2)</f>
+        <v>19.521739130434781</v>
+      </c>
+    </row>
+    <row r="14" spans="1:11" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="H14" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="I14" s="1">
+        <f>I5+K5-2</f>
+        <v>23</v>
+      </c>
+    </row>
+    <row r="15" spans="1:11" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="H15" s="1" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="16" spans="1:11" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="H16" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="I16" s="1">
+        <f>_xlfn.T.INV(I12, I14)</f>
+        <v>-1.7138715277470482</v>
+      </c>
+    </row>
+    <row r="17" spans="8:10" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="H17" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="I17" s="1">
+        <f>(I6-K6)/(I13*SQRT(1/I5+1/K5))</f>
+        <v>0.37642492706467551</v>
+      </c>
+      <c r="J17" s="1" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="18" spans="8:10" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="H18" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="I18" s="1">
+        <f>I12</f>
+        <v>0.05</v>
+      </c>
+    </row>
+    <row r="19" spans="8:10" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="H19" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="I19" s="1">
+        <f>_xlfn.T.DIST(I17, I14, TRUE)</f>
+        <v>0.64497439187835304</v>
+      </c>
+      <c r="J19" s="1" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="21" spans="8:10" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="H21" s="1" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="23" spans="8:10" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="H23" s="1" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="24" spans="8:10" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="H24" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="I24" s="1">
+        <f>_xlfn.T.INV(0.05/2, I14)</f>
+        <v>-2.0686576104190491</v>
+      </c>
+    </row>
+    <row r="25" spans="8:10" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="H25" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="I25" s="1">
+        <f>_xlfn.T.INV(1-0.05/2, I14)</f>
+        <v>2.0686576104190477</v>
+      </c>
+    </row>
+    <row r="27" spans="8:10" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="H27" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="I27" s="1">
+        <f>I6-K6-I25*SQRT(I13)*SQRT(1/I5+1/K5)</f>
+        <v>-0.73140374060559177</v>
+      </c>
+    </row>
+    <row r="28" spans="8:10" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="H28" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="I28" s="1">
+        <f>I6-K6+I25*SQRT(I13)*SQRT(1/I5+1/K5)</f>
+        <v>6.7314037406055913</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+  <drawing r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>